<commit_message>
Add uncapped +1-per-recommendation bonus, additive to the existing peer score
Per user decision: recommended members get a 추천가산점 equal to their
recommendation count (+1 per recommendation, no cap), layered on top of the
existing 동료환산점수 (which stays capped at 4 recommendations = 20%
weight) rather than replacing it. This keeps the weighted peer component
for baseline fairness while letting broadly-recommended members keep
gaining beyond that cap.

계산_순위표 gets a 추천가산점 column (= 추천받은횟수) and
최종점수 = MAX(0, MIN(100, 자가점검 기준점수 + 팀장조정점수 + 추천가산점)).
Verified against a Python shadow calculation.

ranking_dashboard.html mirrors this in computeRowsFromMembers (bonus =
peerCount, added unweighted like the team-lead adjustment) and shows it
transparently in the admin table (읽기전용 "추천가산" column), the
breakdown captions, and the member view's score header — never hidden.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASm5vDh2GYqn8KMpDHWL8G
</commit_message>
<xml_diff>
--- a/performance_review/구성원_배포용/자가점검표_김영희.xlsx
+++ b/performance_review/구성원_배포용/자가점검표_김영희.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -560,12 +560,19 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 담당자 검토 단계에서 팀장이 -10~+10점의 소폭 조정점수를 더할 수 있습니다(자가점수 부풀리기 방지용, 특별한 사유가 없으면 0). 이 조정은 이 개인 파일이 아니라 관리자 워크북/대시보드에서 이뤄집니다.</t>
+          <t xml:space="preserve">  - 동료평가에서 추천을 받으면(동료환산점수 20% 가중치와 별개로) 추천 1회당 +1점의 추천가산점이 상한 없이 최종점수에 더해집니다.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 담당자 검토 단계에서 팀장이 -10~+10점의 소폭 조정점수를 더할 수 있습니다(자가점수 부풀리기 방지용, 특별한 사유가 없으면 0). 이 조정은 이 개인 파일이 아니라 관리자 워크북/대시보드에서 이뤄집니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">  - 완전 오프라인 파일이며, 회신 전까지 본인 PC에만 저장됩니다.</t>
         </is>

</xml_diff>